<commit_message>
vault backup: 2026-07-09 09:25:04
</commit_message>
<xml_diff>
--- a/source/content/Games/AOFS/AOFS Scenarios/AOFS Layout Builder Tool.xlsx
+++ b/source/content/Games/AOFS/AOFS Scenarios/AOFS Layout Builder Tool.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/686448e349e6805c/Desktop/Age Of Fantasy Skirmish/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/686448e349e6805c/Documents/GitHub/Dungeons-And-Dragons/source/content/Games/AOFS/AOFS Scenarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CBF22125-4490-42DE-A2FD-9F5DEA6B2859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{CBF22125-4490-42DE-A2FD-9F5DEA6B2859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A117407-1432-4E63-8BAD-6F1B313369FE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="67740" windowHeight="44520" activeTab="1" xr2:uid="{1B8C7405-B1DB-488B-8B51-388461EF341C}"/>
+    <workbookView minimized="1" xWindow="11190" yWindow="24570" windowWidth="50625" windowHeight="19710" activeTab="3" xr2:uid="{1B8C7405-B1DB-488B-8B51-388461EF341C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blank Grid" sheetId="1" r:id="rId1"/>
     <sheet name="Scenario 1" sheetId="2" r:id="rId2"/>
     <sheet name="Scenario 2" sheetId="3" r:id="rId3"/>
+    <sheet name="Scenario 3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -252,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1441,6 +1442,61 @@
         <a:xfrm>
           <a:off x="8904329" y="10179750"/>
           <a:ext cx="912076" cy="912077"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>581025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>447675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Graphic 1" descr="Badge 1 with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D8EFD90-D262-43C0-845B-DF40071DEDFA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5838825" y="4772025"/>
+          <a:ext cx="914400" cy="914400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2102,4 +2158,115 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{769EFC50-D14D-4B54-9E33-975331D45CF3}">
+  <dimension ref="B1:K9"/>
+  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="82.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="15.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:11" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="11"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="21"/>
+    </row>
+    <row r="3" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="16"/>
+    </row>
+    <row r="4" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="13"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="13"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="16"/>
+    </row>
+    <row r="6" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="13"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="16"/>
+    </row>
+    <row r="7" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="13"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="16"/>
+    </row>
+    <row r="8" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="13"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="16"/>
+    </row>
+    <row r="9" spans="2:11" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="22"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="18"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-08-18 19:13:41
</commit_message>
<xml_diff>
--- a/source/content/Games/AOFS/AOFS Scenarios/AOFS Layout Builder Tool.xlsx
+++ b/source/content/Games/AOFS/AOFS Scenarios/AOFS Layout Builder Tool.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/686448e349e6805c/Documents/GitHub/Dungeons-And-Dragons/source/content/Games/AOFS/AOFS Scenarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{CBF22125-4490-42DE-A2FD-9F5DEA6B2859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A117407-1432-4E63-8BAD-6F1B313369FE}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{CBF22125-4490-42DE-A2FD-9F5DEA6B2859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EF472EB-0CF6-4AAB-8400-1ABAA67EFD31}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="11190" yWindow="24570" windowWidth="50625" windowHeight="19710" activeTab="3" xr2:uid="{1B8C7405-B1DB-488B-8B51-388461EF341C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="67740" windowHeight="44520" activeTab="4" xr2:uid="{1B8C7405-B1DB-488B-8B51-388461EF341C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blank Grid" sheetId="1" r:id="rId1"/>
     <sheet name="Scenario 1" sheetId="2" r:id="rId2"/>
     <sheet name="Scenario 2" sheetId="3" r:id="rId3"/>
     <sheet name="Scenario 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Scenario 4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -85,6 +86,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -233,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -258,6 +271,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1497,6 +1512,261 @@
         <a:xfrm>
           <a:off x="5838825" y="4772025"/>
           <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>583038</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>449688</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Graphic 1" descr="Badge 1 with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{467065B4-387F-4666-976F-38D592E5D9BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5829300" y="4774038"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>83557</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>42822</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>995634</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>954899</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Graphic 2" descr="Badge with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DA7A2A2-AB94-4BB0-A9AC-33C25BEDE1DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3226807" y="3186072"/>
+          <a:ext cx="912077" cy="912077"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>64662</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>979062</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>990600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Graphic 3" descr="Badge 3 with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9ED3C8E-5DF7-46A3-98FA-FD35D4E69A04}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8446662" y="3219450"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>988277</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>978752</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Graphic 4" descr="Badge 4 with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7592EAA6-FFE0-4975-A0D5-DC80FAE9BAC6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId8"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3219450" y="6353175"/>
+          <a:ext cx="912077" cy="912077"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>46154</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>105628</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>958231</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>1017705</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Graphic 5" descr="Badge 5 with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2DA2F43-1F5A-43B3-9FAD-9118C53151C2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId10"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8428154" y="6392128"/>
+          <a:ext cx="912077" cy="912077"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2269,4 +2539,115 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53636CE-38C8-4396-9224-72D51C75A66E}">
+  <dimension ref="B1:K9"/>
+  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="82.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="15.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:11" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="11"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="21"/>
+    </row>
+    <row r="3" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="13"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="16"/>
+    </row>
+    <row r="4" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="13"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="13"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="16"/>
+    </row>
+    <row r="6" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="13"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="16"/>
+    </row>
+    <row r="7" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="13"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="16"/>
+    </row>
+    <row r="8" spans="2:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="13"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="16"/>
+    </row>
+    <row r="9" spans="2:11" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="22"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="18"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>